<commit_message>
Added more documentation and updated some sections
</commit_message>
<xml_diff>
--- a/results/dca_analysis_summary.xlsx
+++ b/results/dca_analysis_summary.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Full Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Error Statistics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Error Ranges" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -597,25 +598,25 @@
         <v>4049454.6</v>
       </c>
       <c r="E4" t="n">
-        <v>1669690.556182475</v>
+        <v>1669690.27338862</v>
       </c>
       <c r="F4" t="n">
-        <v>5719145.156182475</v>
+        <v>5719144.87338862</v>
       </c>
       <c r="G4" t="n">
         <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>21.75182333705217</v>
+        <v>21.75182337274285</v>
       </c>
       <c r="I4" t="n">
-        <v>26.6985810059546</v>
+        <v>26.69858100564651</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1838804058756189</v>
+        <v>0.183880408805129</v>
       </c>
       <c r="K4" t="n">
-        <v>16.40084284333451</v>
+        <v>16.40084413982048</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>34881</v>
@@ -669,7 +670,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hyperbolic</t>
+          <t>Exponential</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -681,25 +682,25 @@
         <v>3644429</v>
       </c>
       <c r="E6" t="n">
-        <v>1894858.094297095</v>
+        <v>1894913.822779634</v>
       </c>
       <c r="F6" t="n">
-        <v>5539287.094297095</v>
+        <v>5539342.822779633</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
       </c>
       <c r="H6" t="n">
-        <v>13.37187437449428</v>
+        <v>13.37259096546025</v>
       </c>
       <c r="I6" t="n">
-        <v>19.31211736747742</v>
+        <v>19.31211745904551</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1797319696819772</v>
+        <v>0.1797469328934891</v>
       </c>
       <c r="K6" t="n">
-        <v>13.43779583710204</v>
+        <v>13.43892744168004</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>32599</v>
@@ -723,25 +724,25 @@
         <v>3172850.1</v>
       </c>
       <c r="E7" t="n">
-        <v>3639378.206649796</v>
+        <v>3639378.235961125</v>
       </c>
       <c r="F7" t="n">
-        <v>6812228.306649795</v>
+        <v>6812228.335961124</v>
       </c>
       <c r="G7" t="n">
         <v>10</v>
       </c>
       <c r="H7" t="n">
-        <v>80.76874945820771</v>
+        <v>80.76874957275557</v>
       </c>
       <c r="I7" t="n">
-        <v>111.867612522504</v>
+        <v>111.8676125225151</v>
       </c>
       <c r="J7" t="n">
-        <v>14.65868970017692</v>
+        <v>14.65868985072408</v>
       </c>
       <c r="K7" t="n">
-        <v>33.21819770301752</v>
+        <v>33.21819776738316</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>26299</v>
@@ -753,7 +754,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Exponential</t>
+          <t>Hyperbolic</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -765,25 +766,25 @@
         <v>3164706.9</v>
       </c>
       <c r="E8" t="n">
-        <v>3259760.423863981</v>
+        <v>3259747.651170223</v>
       </c>
       <c r="F8" t="n">
-        <v>6424467.323863981</v>
+        <v>6424454.551170223</v>
       </c>
       <c r="G8" t="n">
         <v>10</v>
       </c>
       <c r="H8" t="n">
-        <v>38.22117989586559</v>
+        <v>38.15471553678263</v>
       </c>
       <c r="I8" t="n">
-        <v>50.5012185228081</v>
+        <v>50.41289071324042</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3681647865892472</v>
+        <v>0.3681355831463982</v>
       </c>
       <c r="K8" t="n">
-        <v>17.79902866153802</v>
+        <v>17.7796031285808</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>34973</v>
@@ -807,25 +808,25 @@
         <v>2981528</v>
       </c>
       <c r="E9" t="n">
-        <v>1586534.133643676</v>
+        <v>1588150.709538674</v>
       </c>
       <c r="F9" t="n">
-        <v>4568062.133643677</v>
+        <v>4569678.709538674</v>
       </c>
       <c r="G9" t="n">
         <v>10</v>
       </c>
       <c r="H9" t="n">
-        <v>15.71886713997776</v>
+        <v>15.7077437154223</v>
       </c>
       <c r="I9" t="n">
-        <v>21.36598743472548</v>
+        <v>21.3556525243219</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1134954327035107</v>
+        <v>0.1134255224669206</v>
       </c>
       <c r="K9" t="n">
-        <v>10.55435288933695</v>
+        <v>10.54668805079436</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>36342</v>
@@ -849,25 +850,25 @@
         <v>2820640.7</v>
       </c>
       <c r="E10" t="n">
-        <v>2942005.30391826</v>
+        <v>2942005.305977425</v>
       </c>
       <c r="F10" t="n">
-        <v>5762646.00391826</v>
+        <v>5762646.005977426</v>
       </c>
       <c r="G10" t="n">
         <v>10</v>
       </c>
       <c r="H10" t="n">
-        <v>62.95855533844045</v>
+        <v>62.9585553221982</v>
       </c>
       <c r="I10" t="n">
-        <v>85.5321693166338</v>
+        <v>85.53216931663377</v>
       </c>
       <c r="J10" t="n">
-        <v>4.816701419773568</v>
+        <v>4.816701422896827</v>
       </c>
       <c r="K10" t="n">
-        <v>27.91083320451947</v>
+        <v>27.91083319228155</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>37347</v>
@@ -900,7 +901,7 @@
         <v>10</v>
       </c>
       <c r="H11" t="n">
-        <v>68.05951962267997</v>
+        <v>68.05951962267999</v>
       </c>
       <c r="I11" t="n">
         <v>88.14928367003853</v>
@@ -921,7 +922,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Exponential</t>
+          <t>Hyperbolic</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -933,25 +934,25 @@
         <v>1499667.9</v>
       </c>
       <c r="E12" t="n">
-        <v>1667380.046768384</v>
+        <v>1667381.871832623</v>
       </c>
       <c r="F12" t="n">
-        <v>3167047.946768383</v>
+        <v>3167049.771832623</v>
       </c>
       <c r="G12" t="n">
         <v>5</v>
       </c>
       <c r="H12" t="n">
-        <v>34.08451783423458</v>
+        <v>34.08451149305042</v>
       </c>
       <c r="I12" t="n">
-        <v>50.0796491627848</v>
+        <v>50.07964904160279</v>
       </c>
       <c r="J12" t="n">
-        <v>58.1246248869118</v>
+        <v>58.12481928109533</v>
       </c>
       <c r="K12" t="n">
-        <v>28.1023078341604</v>
+        <v>28.10228454834861</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>35977</v>
@@ -975,25 +976,25 @@
         <v>1652248.4</v>
       </c>
       <c r="E13" t="n">
-        <v>2362940.390087321</v>
+        <v>2363101.08938124</v>
       </c>
       <c r="F13" t="n">
-        <v>4015188.790087321</v>
+        <v>4015349.489381241</v>
       </c>
       <c r="G13" t="n">
         <v>5</v>
       </c>
       <c r="H13" t="n">
-        <v>39.96901518108626</v>
+        <v>39.96773779138248</v>
       </c>
       <c r="I13" t="n">
-        <v>51.36455038458232</v>
+        <v>51.36455237750198</v>
       </c>
       <c r="J13" t="n">
-        <v>133.130590441469</v>
+        <v>133.1454329925278</v>
       </c>
       <c r="K13" t="n">
-        <v>25.97700637162984</v>
+        <v>25.97614835293198</v>
       </c>
       <c r="L13" s="2" t="n">
         <v>37073</v>
@@ -1017,25 +1018,25 @@
         <v>504216.4</v>
       </c>
       <c r="E14" t="n">
-        <v>529823.4257940267</v>
+        <v>529823.4251892607</v>
       </c>
       <c r="F14" t="n">
-        <v>1034039.825794027</v>
+        <v>1034039.825189261</v>
       </c>
       <c r="G14" t="n">
         <v>10</v>
       </c>
       <c r="H14" t="n">
-        <v>6.867743902280183</v>
+        <v>6.867743917267984</v>
       </c>
       <c r="I14" t="n">
-        <v>8.968282992939326</v>
+        <v>8.968282992939521</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1080201876361208</v>
+        <v>0.1080201877650492</v>
       </c>
       <c r="K14" t="n">
-        <v>10.35637673844463</v>
+        <v>10.35637676053156</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>40269</v>
@@ -1155,10 +1156,10 @@
         <v>5.754989165801362</v>
       </c>
       <c r="I17" t="n">
-        <v>7.103190214692428</v>
+        <v>7.103190214692429</v>
       </c>
       <c r="J17" t="n">
-        <v>0.09679565752484261</v>
+        <v>0.09679565752484262</v>
       </c>
       <c r="K17" t="n">
         <v>9.349057899207097</v>
@@ -1227,25 +1228,25 @@
         <v>317279.9</v>
       </c>
       <c r="E19" t="n">
-        <v>356442.0617369795</v>
+        <v>356442.0618512596</v>
       </c>
       <c r="F19" t="n">
-        <v>673721.9617369794</v>
+        <v>673721.9618512595</v>
       </c>
       <c r="G19" t="n">
         <v>5</v>
       </c>
       <c r="H19" t="n">
-        <v>2.259247144425327</v>
+        <v>2.259247142610894</v>
       </c>
       <c r="I19" t="n">
-        <v>3.079901818267771</v>
+        <v>3.079901818267772</v>
       </c>
       <c r="J19" t="n">
-        <v>0.04119955730565326</v>
+        <v>0.04119955728669649</v>
       </c>
       <c r="K19" t="n">
-        <v>4.113428483689668</v>
+        <v>4.113428480851155</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>41000</v>
@@ -1269,25 +1270,25 @@
         <v>503296.7</v>
       </c>
       <c r="E20" t="n">
-        <v>519474.9660761253</v>
+        <v>519474.9663830572</v>
       </c>
       <c r="F20" t="n">
-        <v>1022771.666076125</v>
+        <v>1022771.666383057</v>
       </c>
       <c r="G20" t="n">
         <v>15</v>
       </c>
       <c r="H20" t="n">
-        <v>17.74280122283182</v>
+        <v>17.7428012178733</v>
       </c>
       <c r="I20" t="n">
-        <v>22.50375149834873</v>
+        <v>22.50375149834879</v>
       </c>
       <c r="J20" t="n">
-        <v>0.513777800006442</v>
+        <v>0.5137778008524776</v>
       </c>
       <c r="K20" t="n">
-        <v>31.1263118207892</v>
+        <v>31.1263118212506</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>41000</v>
@@ -1437,25 +1438,25 @@
         <v>1728594.7</v>
       </c>
       <c r="E24" t="n">
-        <v>1781174.365867433</v>
+        <v>1781174.365859224</v>
       </c>
       <c r="F24" t="n">
-        <v>3509769.065867433</v>
+        <v>3509769.065859224</v>
       </c>
       <c r="G24" t="n">
         <v>10</v>
       </c>
       <c r="H24" t="n">
-        <v>32.81577294986901</v>
+        <v>32.81577294947356</v>
       </c>
       <c r="I24" t="n">
         <v>41.56344569009644</v>
       </c>
       <c r="J24" t="n">
-        <v>1.940956207148876</v>
+        <v>1.940956207163554</v>
       </c>
       <c r="K24" t="n">
-        <v>34.47476187094832</v>
+        <v>34.4747618706435</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>37712</v>
@@ -1479,25 +1480,25 @@
         <v>1649685.9</v>
       </c>
       <c r="E25" t="n">
-        <v>860572.8366778082</v>
+        <v>860572.8341329525</v>
       </c>
       <c r="F25" t="n">
-        <v>2510258.736677809</v>
+        <v>2510258.734132953</v>
       </c>
       <c r="G25" t="n">
         <v>10</v>
       </c>
       <c r="H25" t="n">
-        <v>17.71868566191207</v>
+        <v>17.71868561784895</v>
       </c>
       <c r="I25" t="n">
-        <v>25.45655630888686</v>
+        <v>25.45655630888714</v>
       </c>
       <c r="J25" t="n">
-        <v>0.2819307227486246</v>
+        <v>0.2819307204093798</v>
       </c>
       <c r="K25" t="n">
-        <v>23.4515259792096</v>
+        <v>23.45152586050902</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>34060</v>
@@ -1521,25 +1522,25 @@
         <v>1258481.7</v>
       </c>
       <c r="E26" t="n">
-        <v>1312014.919656853</v>
+        <v>1312014.951175399</v>
       </c>
       <c r="F26" t="n">
-        <v>2570496.619656853</v>
+        <v>2570496.651175399</v>
       </c>
       <c r="G26" t="n">
         <v>10</v>
       </c>
       <c r="H26" t="n">
-        <v>18.31001296326223</v>
+        <v>18.31001298564336</v>
       </c>
       <c r="I26" t="n">
-        <v>24.43560867639657</v>
+        <v>24.43560867639697</v>
       </c>
       <c r="J26" t="n">
-        <v>3.329098541673174</v>
+        <v>3.329098882073747</v>
       </c>
       <c r="K26" t="n">
-        <v>20.09252099139783</v>
+        <v>20.09251922979521</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>35886</v>
@@ -1563,25 +1564,25 @@
         <v>1203326.1</v>
       </c>
       <c r="E27" t="n">
-        <v>2092927.367396122</v>
+        <v>2092927.487986102</v>
       </c>
       <c r="F27" t="n">
-        <v>3296253.467396122</v>
+        <v>3296253.587986102</v>
       </c>
       <c r="G27" t="n">
         <v>5</v>
       </c>
       <c r="H27" t="n">
-        <v>45.83075063891995</v>
+        <v>45.8307506825978</v>
       </c>
       <c r="I27" t="n">
-        <v>56.29978400719518</v>
+        <v>56.29978400716741</v>
       </c>
       <c r="J27" t="n">
-        <v>0.9018323990543069</v>
+        <v>0.9018324006269297</v>
       </c>
       <c r="K27" t="n">
-        <v>31.17606605576583</v>
+        <v>31.17606602490879</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>39173</v>
@@ -1605,25 +1606,25 @@
         <v>1162915.7</v>
       </c>
       <c r="E28" t="n">
-        <v>1349388.928167786</v>
+        <v>1349388.901466775</v>
       </c>
       <c r="F28" t="n">
-        <v>2512304.628167787</v>
+        <v>2512304.601466775</v>
       </c>
       <c r="G28" t="n">
         <v>5</v>
       </c>
       <c r="H28" t="n">
-        <v>36.19178813572185</v>
+        <v>36.19178779832809</v>
       </c>
       <c r="I28" t="n">
-        <v>48.62122899931555</v>
+        <v>48.62122899930931</v>
       </c>
       <c r="J28" t="n">
-        <v>4.608923061251133</v>
+        <v>4.608923020697977</v>
       </c>
       <c r="K28" t="n">
-        <v>32.972381367095</v>
+        <v>32.97238135960348</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>39264</v>
@@ -1689,25 +1690,25 @@
         <v>1152533.7</v>
       </c>
       <c r="E30" t="n">
-        <v>680791.2792104975</v>
+        <v>680791.278197408</v>
       </c>
       <c r="F30" t="n">
-        <v>1833324.979210497</v>
+        <v>1833324.978197408</v>
       </c>
       <c r="G30" t="n">
         <v>2</v>
       </c>
       <c r="H30" t="n">
-        <v>4.640056253771625</v>
+        <v>4.640056244026986</v>
       </c>
       <c r="I30" t="n">
-        <v>7.273433098560717</v>
+        <v>7.273433098560473</v>
       </c>
       <c r="J30" t="n">
-        <v>0.1645264439593898</v>
+        <v>0.164526443456749</v>
       </c>
       <c r="K30" t="n">
-        <v>13.43241340255312</v>
+        <v>13.43241336584211</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>33329</v>
@@ -1775,16 +1776,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35.05629198006821</v>
+        <v>35.05359697638244</v>
       </c>
       <c r="C3" t="n">
-        <v>46.02403197181918</v>
+        <v>46.02062987675034</v>
       </c>
       <c r="D3" t="n">
-        <v>8.093674661102604</v>
+        <v>8.094190290444782</v>
       </c>
       <c r="E3" t="n">
-        <v>20.42373408324815</v>
+        <v>20.42280854329037</v>
       </c>
     </row>
     <row r="4">
@@ -1794,16 +1795,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48.54081370172421</v>
+        <v>48.54080274567475</v>
       </c>
       <c r="C4" t="n">
-        <v>60.97745958273973</v>
+        <v>60.97737944346766</v>
       </c>
       <c r="D4" t="n">
-        <v>26.3998388450528</v>
+        <v>26.40236358202489</v>
       </c>
       <c r="E4" t="n">
-        <v>10.97444054438078</v>
+        <v>10.974811486458</v>
       </c>
     </row>
     <row r="5">
@@ -1838,10 +1839,10 @@
         <v>7.466222178081654</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1134954327035107</v>
+        <v>0.1134255224669206</v>
       </c>
       <c r="E6" t="n">
-        <v>10.55435288933695</v>
+        <v>10.54668805079436</v>
       </c>
     </row>
     <row r="7">
@@ -1851,16 +1852,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18.31001296326223</v>
+        <v>18.31001298564336</v>
       </c>
       <c r="C7" t="n">
-        <v>25.45655630888686</v>
+        <v>25.45655630888714</v>
       </c>
       <c r="D7" t="n">
         <v>0.3543023008289188</v>
       </c>
       <c r="E7" t="n">
-        <v>20.09252099139783</v>
+        <v>20.09251922979521</v>
       </c>
     </row>
     <row r="8">
@@ -1870,13 +1871,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>39.96901518108626</v>
+        <v>39.96773779138248</v>
       </c>
       <c r="C8" t="n">
-        <v>51.36455038458232</v>
+        <v>51.36455237750198</v>
       </c>
       <c r="D8" t="n">
-        <v>3.329098541673174</v>
+        <v>3.329098882073747</v>
       </c>
       <c r="E8" t="n">
         <v>29.1259397358875</v>
@@ -1895,10 +1896,122 @@
         <v>313.3558560067333</v>
       </c>
       <c r="D9" t="n">
-        <v>133.130590441469</v>
+        <v>133.1454329925278</v>
       </c>
       <c r="E9" t="n">
         <v>42.1202591113831</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.137660274749211</v>
+      </c>
+      <c r="C2" t="n">
+        <v>252.3966117119842</v>
+      </c>
+      <c r="D2" t="n">
+        <v>251.258951437235</v>
+      </c>
+      <c r="E2" t="n">
+        <v>18.31001298564336</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.488178940462683</v>
+      </c>
+      <c r="C3" t="n">
+        <v>313.3558560067333</v>
+      </c>
+      <c r="D3" t="n">
+        <v>311.8676770662706</v>
+      </c>
+      <c r="E3" t="n">
+        <v>25.45655630888714</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>MAPE</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.02221975095828346</v>
+      </c>
+      <c r="C4" t="n">
+        <v>133.1454329925278</v>
+      </c>
+      <c r="D4" t="n">
+        <v>133.1232132415695</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.3543023008289188</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>SMAPE</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.219209503439244</v>
+      </c>
+      <c r="C5" t="n">
+        <v>42.1202591113831</v>
+      </c>
+      <c r="D5" t="n">
+        <v>39.90104960794385</v>
+      </c>
+      <c r="E5" t="n">
+        <v>20.09251922979521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>